<commit_message>
ETL Code Logic Rehaul
</commit_message>
<xml_diff>
--- a/Reports/Cleaned/ATWQ12025.xlsx
+++ b/Reports/Cleaned/ATWQ12025.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -434,75 +434,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-03-31 00:00:00</t>
+          <t>InstitutionsLoans</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-12-31 00:00:00</t>
+          <t>45 485 824</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>loans &amp; receivables to credit institutions at amortised cost</t>
+          <t>48 692 644</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>45 485 824</t>
+          <t>CustomersLoans</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>48 692 644</t>
+          <t>418 635 707</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>loans &amp; receivables to customers at amortised cost</t>
+          <t>413 590 717</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>418 635 707</t>
+          <t>TotalAssets</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>413 590 717</t>
+          <t>732 199 134</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
-        <is>
-          <t>total assets</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>732 199 134</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
         <is>
           <t>726 492 948</t>
         </is>
@@ -519,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -535,96 +521,82 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-03-31 00:00:00</t>
+          <t>InstitutionsCredit</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-12-31 00:00:00</t>
+          <t>60 343 286</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>deposits from credit institutions</t>
+          <t>58 977 903</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>60 343 286</t>
+          <t>CustomersCredit</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>58 977 903</t>
+          <t>478 121 800</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>deposits from customers</t>
+          <t>480 478 661</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>478 121 800</t>
+          <t>PrivateEquity</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>480 478 661</t>
+          <t>76 230 841</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>shareholders' equity</t>
+          <t>72 502 834</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>76 230 841</t>
+          <t>TotalLiabilities</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>72 502 834</t>
+          <t>732 199 134</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
-        <is>
-          <t>total liabilities</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>732 199 134</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
         <is>
           <t>726 492 948</t>
         </is>
@@ -641,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -657,75 +629,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-03-31 00:00:00</t>
+          <t>NetBankingIncome</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-03-31 00:00:00</t>
+          <t>9 024 341</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>net banking income</t>
+          <t>8 520 243</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>9 024 341</t>
+          <t>OperatingExpenses</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8 520 243</t>
+          <t>-2 736 814</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>net operating income</t>
+          <t>-2 670 566</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5 026 934</t>
+          <t>NetIncome</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4 488 796</t>
+          <t>3 318 987</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
-        <is>
-          <t>net income</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>3 318 987</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
         <is>
           <t>2 892 578</t>
         </is>
@@ -742,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -758,75 +716,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-03-31 00:00:00</t>
+          <t>InstitutionsLoans</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-12-31 00:00:00</t>
+          <t>45 913 642</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>loans and advances to credit institutions and similar establishments</t>
+          <t>45 580 416</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>45 913 642</t>
+          <t>CustomersLoans</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>45 580 416</t>
+          <t>278 584 476</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>loans and advances to customers</t>
+          <t>271 414 638</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>278 584 476</t>
+          <t>TotalAssets</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>271 414 638</t>
+          <t>482 243 715</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
-        <is>
-          <t>total assets</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>482 243 715</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
         <is>
           <t>482 129 974</t>
         </is>
@@ -843,7 +787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -859,75 +803,82 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-03-31 00:00:00</t>
+          <t>InstitutionsCredit</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-12-31 00:00:00</t>
+          <t>49 636 978</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>amounts owing to credit institutions and similar establishments</t>
+          <t>52 060 161</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>49 636 978</t>
+          <t>CustomersCredit</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>52 060 161</t>
+          <t>337 665 402</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>customer deposits</t>
+          <t>334 753 563</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>337 665 402</t>
+          <t>PrivateEquity</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>334 753 563</t>
+          <t>2 151 408</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>total liabilities</t>
+          <t>2 151 408</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>482 243 715</t>
+          <t>TotalLiabilities</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>482 243 715</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>482 129 974</t>
         </is>
@@ -944,7 +895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -960,75 +911,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-03-31 00:00:00</t>
+          <t>NetBankingIncome</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-03-31 00:00:00</t>
+          <t>5 540 836</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>net banking income</t>
+          <t>4 821 749</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>5 540 836</t>
+          <t>OperatingExpenses</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4 821 749</t>
+          <t>1 360 561</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>operating expenses</t>
+          <t>1 288 438</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1 360 561</t>
+          <t>NetIncome</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1 288 438</t>
+          <t>2 521 388</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
-        <is>
-          <t>net income for the financial year</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2 521 388</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
         <is>
           <t>2 182 953</t>
         </is>

</xml_diff>

<commit_message>
ETL Logic Working Perfectly
</commit_message>
<xml_diff>
--- a/Reports/Cleaned/ATWQ12025.xlsx
+++ b/Reports/Cleaned/ATWQ12025.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -434,61 +434,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>InstitutionsLoans</t>
+          <t>2025-03-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>45 485 824</t>
+          <t>2024-12-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>48 692 644</t>
+          <t>InstitutionsLoans</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CustomersLoans</t>
+          <t>45 485 824</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>418 635 707</t>
+          <t>48 692 644</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>413 590 717</t>
+          <t>CustomersLoans</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TotalAssets</t>
+          <t>418 635 707</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>732 199 134</t>
+          <t>413 590 717</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>TotalAssets</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>732 199 134</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>726 492 948</t>
         </is>
@@ -505,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -521,82 +535,96 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>InstitutionsCredit</t>
+          <t>2025-03-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>60 343 286</t>
+          <t>2024-12-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>58 977 903</t>
+          <t>InstitutionsCredit</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CustomersCredit</t>
+          <t>60 343 286</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>478 121 800</t>
+          <t>58 977 903</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>480 478 661</t>
+          <t>CustomersCredit</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PrivateEquity</t>
+          <t>478 121 800</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>76 230 841</t>
+          <t>480 478 661</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>72 502 834</t>
+          <t>PrivateEquity</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TotalLiabilities</t>
+          <t>76 230 841</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>732 199 134</t>
+          <t>72 502 834</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>TotalLiabilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>732 199 134</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>726 492 948</t>
         </is>
@@ -613,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -629,61 +657,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NetBankingIncome</t>
+          <t>2025-03-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>9 024 341</t>
+          <t>2024-03-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>8 520 243</t>
+          <t>NetBankingIncome</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>OperatingExpenses</t>
+          <t>9 024 341</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>-2 736 814</t>
+          <t>8 520 243</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>-2 670 566</t>
+          <t>OperatingExpenses</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NetIncome</t>
+          <t>-2 736 814</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3 318 987</t>
+          <t>-2 670 566</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>NetIncome</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>3 318 987</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>2 892 578</t>
         </is>
@@ -700,7 +742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -716,61 +758,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>InstitutionsLoans</t>
+          <t>2025-03-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>45 913 642</t>
+          <t>2024-12-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>45 580 416</t>
+          <t>InstitutionsLoans</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CustomersLoans</t>
+          <t>45 913 642</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>278 584 476</t>
+          <t>45 580 416</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>271 414 638</t>
+          <t>CustomersLoans</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TotalAssets</t>
+          <t>278 584 476</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>482 243 715</t>
+          <t>271 414 638</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>TotalAssets</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>482 243 715</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>482 129 974</t>
         </is>
@@ -787,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -803,82 +859,96 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>InstitutionsCredit</t>
+          <t>2025-03-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>49 636 978</t>
+          <t>2024-12-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>52 060 161</t>
+          <t>InstitutionsCredit</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CustomersCredit</t>
+          <t>49 636 978</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>337 665 402</t>
+          <t>52 060 161</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>334 753 563</t>
+          <t>CustomersCredit</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PrivateEquity</t>
+          <t>337 665 402</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2 151 408</t>
+          <t>334 753 563</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2 151 408</t>
+          <t>PrivateEquity</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TotalLiabilities</t>
+          <t>2 151 408</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>482 243 715</t>
+          <t>2 151 408</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>TotalLiabilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>482 243 715</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>482 129 974</t>
         </is>
@@ -895,7 +965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -911,61 +981,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NetBankingIncome</t>
+          <t>2025-03-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5 540 836</t>
+          <t>2024-03-31 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>4 821 749</t>
+          <t>NetBankingIncome</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>OperatingExpenses</t>
+          <t>5 540 836</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1 360 561</t>
+          <t>4 821 749</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1 288 438</t>
+          <t>OperatingExpenses</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NetIncome</t>
+          <t>1 360 561</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2 521 388</t>
+          <t>1 288 438</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>NetIncome</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2 521 388</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>2 182 953</t>
         </is>

</xml_diff>